<commit_message>
docs(seed): regenerate the layout workbook with the AEP/ISP split
Catches the committed workbook up to the generator and the database: 160 items
(was 158) and 34 container configs (was 32), with 19320-6A0 -A510 and
19410-6A0 -A000 each split into their -AEP and -ISP variants.

The two new ISP rows are off-site like their AEP siblings, so Unmatched goes
13 -> 15: they carry a packing rule but no route or eligibility until the
missing plant-hierarchy lines exist.
</commit_message>
<xml_diff>
--- a/reference/MPP_Seed_Layout_Proposal.xlsx
+++ b/reference/MPP_Seed_Layout_Proposal.xlsx
@@ -18,13 +18,13 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$C$26</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Items'!$A$1:$Q$159</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Items'!$A$1:$Q$161</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Eligibility'!$A$1:$F$397</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Routes'!$A$1:$F$377</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'BOMs'!$A$1:$H$155</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Packaging'!$A$1:$J$33</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Unmatched'!$A$1:$F$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'DataIssues'!$A$1:$E$65</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Packaging'!$A$1:$J$35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Unmatched'!$A$1:$F$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'DataIssues'!$A$1:$E$67</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -539,7 +539,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>158 items</t>
+          <t>160 items</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr"/>
@@ -551,7 +551,7 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
@@ -646,7 +646,7 @@
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
@@ -666,11 +666,11 @@
         </is>
       </c>
       <c r="B15" s="2" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>See Unmatched tab - 12 are off-site</t>
+          <t>See Unmatched tab - 14 are off-site</t>
         </is>
       </c>
     </row>
@@ -681,11 +681,11 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>17 HIGH / 35 MED / 12 LOW</t>
+          <t>13 HIGH / 39 MED / 14 LOW</t>
         </is>
       </c>
     </row>
@@ -851,7 +851,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q159"/>
+  <dimension ref="A1:Q161"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -8725,7 +8725,7 @@
     <row r="124">
       <c r="A124" s="3" t="inlineStr">
         <is>
-          <t>19320-6A0 -A510</t>
+          <t>19320-6A0 -A510-AEP</t>
         </is>
       </c>
       <c r="B124" s="3" t="inlineStr">
@@ -8750,7 +8750,7 @@
       </c>
       <c r="F124" s="3" t="inlineStr">
         <is>
-          <t>6AO/6A0</t>
+          <t>6AO</t>
         </is>
       </c>
       <c r="G124" s="3" t="inlineStr">
@@ -8792,12 +8792,12 @@
     <row r="125">
       <c r="A125" s="3" t="inlineStr">
         <is>
-          <t>19410-6A0 -A000</t>
+          <t>19320-6A0 -A510-ISP</t>
         </is>
       </c>
       <c r="B125" s="3" t="inlineStr">
         <is>
-          <t>6A0 Water Passage (AEP)</t>
+          <t>6A0 Thermo Case Auto (ISP)</t>
         </is>
       </c>
       <c r="C125" s="3" t="inlineStr">
@@ -8829,7 +8829,7 @@
       <c r="I125" s="3" t="inlineStr"/>
       <c r="J125" s="3" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>6</t>
         </is>
       </c>
       <c r="K125" s="3" t="inlineStr"/>
@@ -8859,12 +8859,12 @@
     <row r="126">
       <c r="A126" s="3" t="inlineStr">
         <is>
-          <t>19321-64S -A000</t>
+          <t>19410-6A0 -A000-AEP</t>
         </is>
       </c>
       <c r="B126" s="3" t="inlineStr">
         <is>
-          <t>64S Thermo Case</t>
+          <t>6A0 Water Passage (AEP)</t>
         </is>
       </c>
       <c r="C126" s="3" t="inlineStr">
@@ -8884,7 +8884,7 @@
       </c>
       <c r="F126" s="3" t="inlineStr">
         <is>
-          <t>64S</t>
+          <t>6A0</t>
         </is>
       </c>
       <c r="G126" s="3" t="inlineStr">
@@ -8896,7 +8896,7 @@
       <c r="I126" s="3" t="inlineStr"/>
       <c r="J126" s="3" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>60</t>
         </is>
       </c>
       <c r="K126" s="3" t="inlineStr"/>
@@ -8926,12 +8926,12 @@
     <row r="127">
       <c r="A127" s="3" t="inlineStr">
         <is>
-          <t>12270-6MA -J000</t>
+          <t>19410-6A0 -A000-ISP</t>
         </is>
       </c>
       <c r="B127" s="3" t="inlineStr">
         <is>
-          <t>6MA Fuel Pump</t>
+          <t>6A0 Water Passage (ISP)</t>
         </is>
       </c>
       <c r="C127" s="3" t="inlineStr">
@@ -8951,7 +8951,7 @@
       </c>
       <c r="F127" s="3" t="inlineStr">
         <is>
-          <t>6MA</t>
+          <t>6A0</t>
         </is>
       </c>
       <c r="G127" s="3" t="inlineStr">
@@ -8963,7 +8963,7 @@
       <c r="I127" s="3" t="inlineStr"/>
       <c r="J127" s="3" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>15</t>
         </is>
       </c>
       <c r="K127" s="3" t="inlineStr"/>
@@ -8993,12 +8993,12 @@
     <row r="128">
       <c r="A128" s="3" t="inlineStr">
         <is>
-          <t>19321-66V -A000</t>
+          <t>19321-64S -A000</t>
         </is>
       </c>
       <c r="B128" s="3" t="inlineStr">
         <is>
-          <t>66V Thermo Case</t>
+          <t>64S Thermo Case</t>
         </is>
       </c>
       <c r="C128" s="3" t="inlineStr">
@@ -9018,7 +9018,7 @@
       </c>
       <c r="F128" s="3" t="inlineStr">
         <is>
-          <t>66V</t>
+          <t>64S</t>
         </is>
       </c>
       <c r="G128" s="3" t="inlineStr">
@@ -9060,12 +9060,12 @@
     <row r="129">
       <c r="A129" s="3" t="inlineStr">
         <is>
-          <t>12270-6MD -A000</t>
+          <t>12270-6MA -J000</t>
         </is>
       </c>
       <c r="B129" s="3" t="inlineStr">
         <is>
-          <t>6MD Fuel Pump</t>
+          <t>6MA Fuel Pump</t>
         </is>
       </c>
       <c r="C129" s="3" t="inlineStr">
@@ -9085,7 +9085,7 @@
       </c>
       <c r="F129" s="3" t="inlineStr">
         <is>
-          <t>6MD</t>
+          <t>6MA</t>
         </is>
       </c>
       <c r="G129" s="3" t="inlineStr">
@@ -9127,12 +9127,12 @@
     <row r="130">
       <c r="A130" s="3" t="inlineStr">
         <is>
-          <t>14850-6MD -A000</t>
+          <t>19321-66V -A000</t>
         </is>
       </c>
       <c r="B130" s="3" t="inlineStr">
         <is>
-          <t>6MD Oil Jet</t>
+          <t>66V Thermo Case</t>
         </is>
       </c>
       <c r="C130" s="3" t="inlineStr">
@@ -9152,7 +9152,7 @@
       </c>
       <c r="F130" s="3" t="inlineStr">
         <is>
-          <t>6MD</t>
+          <t>66V</t>
         </is>
       </c>
       <c r="G130" s="3" t="inlineStr">
@@ -9164,7 +9164,7 @@
       <c r="I130" s="3" t="inlineStr"/>
       <c r="J130" s="3" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>6</t>
         </is>
       </c>
       <c r="K130" s="3" t="inlineStr"/>
@@ -9194,12 +9194,12 @@
     <row r="131">
       <c r="A131" s="3" t="inlineStr">
         <is>
-          <t>19410-6MD -A000</t>
+          <t>12270-6MD -A000</t>
         </is>
       </c>
       <c r="B131" s="3" t="inlineStr">
         <is>
-          <t>6MD Water Passage</t>
+          <t>6MD Fuel Pump</t>
         </is>
       </c>
       <c r="C131" s="3" t="inlineStr">
@@ -9231,7 +9231,7 @@
       <c r="I131" s="3" t="inlineStr"/>
       <c r="J131" s="3" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>10</t>
         </is>
       </c>
       <c r="K131" s="3" t="inlineStr"/>
@@ -9261,12 +9261,12 @@
     <row r="132">
       <c r="A132" s="3" t="inlineStr">
         <is>
-          <t>12230-P8A -A000</t>
+          <t>14850-6MD -A000</t>
         </is>
       </c>
       <c r="B132" s="3" t="inlineStr">
         <is>
-          <t>Cam Thrust Front</t>
+          <t>6MD Oil Jet</t>
         </is>
       </c>
       <c r="C132" s="3" t="inlineStr">
@@ -9286,7 +9286,7 @@
       </c>
       <c r="F132" s="3" t="inlineStr">
         <is>
-          <t>P8A</t>
+          <t>6MD</t>
         </is>
       </c>
       <c r="G132" s="3" t="inlineStr">
@@ -9298,7 +9298,7 @@
       <c r="I132" s="3" t="inlineStr"/>
       <c r="J132" s="3" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>60</t>
         </is>
       </c>
       <c r="K132" s="3" t="inlineStr"/>
@@ -9328,12 +9328,12 @@
     <row r="133">
       <c r="A133" s="3" t="inlineStr">
         <is>
-          <t>19321-66V-A100</t>
+          <t>19410-6MD -A000</t>
         </is>
       </c>
       <c r="B133" s="3" t="inlineStr">
         <is>
-          <t>66V Thermo Case</t>
+          <t>6MD Water Passage</t>
         </is>
       </c>
       <c r="C133" s="3" t="inlineStr">
@@ -9353,7 +9353,7 @@
       </c>
       <c r="F133" s="3" t="inlineStr">
         <is>
-          <t>66V</t>
+          <t>6MD</t>
         </is>
       </c>
       <c r="G133" s="3" t="inlineStr">
@@ -9365,7 +9365,7 @@
       <c r="I133" s="3" t="inlineStr"/>
       <c r="J133" s="3" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>60</t>
         </is>
       </c>
       <c r="K133" s="3" t="inlineStr"/>
@@ -9393,148 +9393,148 @@
       <c r="Q133" s="3" t="inlineStr"/>
     </row>
     <row r="134">
-      <c r="A134" s="4" t="inlineStr">
-        <is>
-          <t>12231-RPY -G000-M</t>
-        </is>
-      </c>
-      <c r="B134" s="4" t="inlineStr">
-        <is>
-          <t>RPY Cam Holder In #1 (machined)</t>
-        </is>
-      </c>
-      <c r="C134" s="4" t="inlineStr">
-        <is>
-          <t>SubAssembly</t>
-        </is>
-      </c>
-      <c r="D134" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E134" s="4" t="inlineStr">
-        <is>
-          <t>Machined</t>
-        </is>
-      </c>
-      <c r="F134" s="4" t="inlineStr">
-        <is>
-          <t>RPY/5BA</t>
-        </is>
-      </c>
-      <c r="G134" s="4" t="inlineStr">
+      <c r="A134" s="3" t="inlineStr">
+        <is>
+          <t>12230-P8A -A000</t>
+        </is>
+      </c>
+      <c r="B134" s="3" t="inlineStr">
+        <is>
+          <t>Cam Thrust Front</t>
+        </is>
+      </c>
+      <c r="C134" s="3" t="inlineStr">
+        <is>
+          <t>FinishedGood</t>
+        </is>
+      </c>
+      <c r="D134" s="3" t="inlineStr">
+        <is>
+          <t>FinishedGood</t>
+        </is>
+      </c>
+      <c r="E134" s="3" t="inlineStr">
+        <is>
+          <t>Assembled</t>
+        </is>
+      </c>
+      <c r="F134" s="3" t="inlineStr">
+        <is>
+          <t>P8A</t>
+        </is>
+      </c>
+      <c r="G134" s="3" t="inlineStr">
         <is>
           <t>EA</t>
         </is>
       </c>
-      <c r="H134" s="4" t="inlineStr"/>
-      <c r="I134" s="4" t="inlineStr"/>
-      <c r="J134" s="4" t="inlineStr"/>
-      <c r="K134" s="4" t="inlineStr"/>
-      <c r="L134" s="4" t="inlineStr"/>
-      <c r="M134" s="4" t="inlineStr">
-        <is>
-          <t>Blue Ridge (synthesized)</t>
-        </is>
-      </c>
-      <c r="N134" s="4" t="inlineStr">
+      <c r="H134" s="3" t="inlineStr"/>
+      <c r="I134" s="3" t="inlineStr"/>
+      <c r="J134" s="3" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="K134" s="3" t="inlineStr"/>
+      <c r="L134" s="3" t="inlineStr"/>
+      <c r="M134" s="3" t="inlineStr">
+        <is>
+          <t>Off-Site</t>
+        </is>
+      </c>
+      <c r="N134" s="3" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="O134" s="4" t="inlineStr">
-        <is>
-          <t>MA2-RPY6B2, MA2-RPYCAM1, MA2-RPYCAM2</t>
-        </is>
-      </c>
-      <c r="P134" s="4" t="inlineStr">
-        <is>
-          <t>SYNTHESIZED</t>
-        </is>
-      </c>
-      <c r="Q134" s="4" t="inlineStr">
-        <is>
-          <t>Machined identity minted by Machining OUT from 12231-RPY -G000.</t>
-        </is>
-      </c>
+      <c r="O134" s="3" t="inlineStr">
+        <is>
+          <t>(none)</t>
+        </is>
+      </c>
+      <c r="P134" s="3" t="inlineStr">
+        <is>
+          <t>OFF-SITE</t>
+        </is>
+      </c>
+      <c r="Q134" s="3" t="inlineStr"/>
     </row>
     <row r="135">
-      <c r="A135" s="4" t="inlineStr">
-        <is>
-          <t>12232-RPY -G000-M</t>
-        </is>
-      </c>
-      <c r="B135" s="4" t="inlineStr">
-        <is>
-          <t>RPY Cam Holder In #2 (machined)</t>
-        </is>
-      </c>
-      <c r="C135" s="4" t="inlineStr">
-        <is>
-          <t>SubAssembly</t>
-        </is>
-      </c>
-      <c r="D135" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E135" s="4" t="inlineStr">
-        <is>
-          <t>Machined</t>
-        </is>
-      </c>
-      <c r="F135" s="4" t="inlineStr">
-        <is>
-          <t>RPY/5BA</t>
-        </is>
-      </c>
-      <c r="G135" s="4" t="inlineStr">
+      <c r="A135" s="3" t="inlineStr">
+        <is>
+          <t>19321-66V-A100</t>
+        </is>
+      </c>
+      <c r="B135" s="3" t="inlineStr">
+        <is>
+          <t>66V Thermo Case</t>
+        </is>
+      </c>
+      <c r="C135" s="3" t="inlineStr">
+        <is>
+          <t>FinishedGood</t>
+        </is>
+      </c>
+      <c r="D135" s="3" t="inlineStr">
+        <is>
+          <t>FinishedGood</t>
+        </is>
+      </c>
+      <c r="E135" s="3" t="inlineStr">
+        <is>
+          <t>Assembled</t>
+        </is>
+      </c>
+      <c r="F135" s="3" t="inlineStr">
+        <is>
+          <t>66V</t>
+        </is>
+      </c>
+      <c r="G135" s="3" t="inlineStr">
         <is>
           <t>EA</t>
         </is>
       </c>
-      <c r="H135" s="4" t="inlineStr"/>
-      <c r="I135" s="4" t="inlineStr"/>
-      <c r="J135" s="4" t="inlineStr"/>
-      <c r="K135" s="4" t="inlineStr"/>
-      <c r="L135" s="4" t="inlineStr"/>
-      <c r="M135" s="4" t="inlineStr">
-        <is>
-          <t>Blue Ridge (synthesized)</t>
-        </is>
-      </c>
-      <c r="N135" s="4" t="inlineStr">
+      <c r="H135" s="3" t="inlineStr"/>
+      <c r="I135" s="3" t="inlineStr"/>
+      <c r="J135" s="3" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="K135" s="3" t="inlineStr"/>
+      <c r="L135" s="3" t="inlineStr"/>
+      <c r="M135" s="3" t="inlineStr">
+        <is>
+          <t>Off-Site</t>
+        </is>
+      </c>
+      <c r="N135" s="3" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="O135" s="4" t="inlineStr">
-        <is>
-          <t>MA2-RPY6B2, MA2-RPYCAM1, MA2-RPYCAM2</t>
-        </is>
-      </c>
-      <c r="P135" s="4" t="inlineStr">
-        <is>
-          <t>SYNTHESIZED</t>
-        </is>
-      </c>
-      <c r="Q135" s="4" t="inlineStr">
-        <is>
-          <t>Machined identity minted by Machining OUT from 12232-RPY -G000.</t>
-        </is>
-      </c>
+      <c r="O135" s="3" t="inlineStr">
+        <is>
+          <t>(none)</t>
+        </is>
+      </c>
+      <c r="P135" s="3" t="inlineStr">
+        <is>
+          <t>OFF-SITE</t>
+        </is>
+      </c>
+      <c r="Q135" s="3" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" s="4" t="inlineStr">
         <is>
-          <t>12233-RPY -G000-M</t>
+          <t>12231-RPY -G000-M</t>
         </is>
       </c>
       <c r="B136" s="4" t="inlineStr">
         <is>
-          <t>RPY Cam Holder In #3 (machined)</t>
+          <t>RPY Cam Holder In #1 (machined)</t>
         </is>
       </c>
       <c r="C136" s="4" t="inlineStr">
@@ -9589,19 +9589,19 @@
       </c>
       <c r="Q136" s="4" t="inlineStr">
         <is>
-          <t>Machined identity minted by Machining OUT from 12233-RPY -G000.</t>
+          <t>Machined identity minted by Machining OUT from 12231-RPY -G000.</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="4" t="inlineStr">
         <is>
-          <t>12234-RPY -G000-M</t>
+          <t>12232-RPY -G000-M</t>
         </is>
       </c>
       <c r="B137" s="4" t="inlineStr">
         <is>
-          <t>RPY Cam Holder In #4 (machined)</t>
+          <t>RPY Cam Holder In #2 (machined)</t>
         </is>
       </c>
       <c r="C137" s="4" t="inlineStr">
@@ -9656,19 +9656,19 @@
       </c>
       <c r="Q137" s="4" t="inlineStr">
         <is>
-          <t>Machined identity minted by Machining OUT from 12234-RPY -G000.</t>
+          <t>Machined identity minted by Machining OUT from 12232-RPY -G000.</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="4" t="inlineStr">
         <is>
-          <t>12235-RPY -G000-M</t>
+          <t>12233-RPY -G000-M</t>
         </is>
       </c>
       <c r="B138" s="4" t="inlineStr">
         <is>
-          <t>RPY Cam Holder In #5 (machined)</t>
+          <t>RPY Cam Holder In #3 (machined)</t>
         </is>
       </c>
       <c r="C138" s="4" t="inlineStr">
@@ -9723,19 +9723,19 @@
       </c>
       <c r="Q138" s="4" t="inlineStr">
         <is>
-          <t>Machined identity minted by Machining OUT from 12235-RPY -G000.</t>
+          <t>Machined identity minted by Machining OUT from 12233-RPY -G000.</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="4" t="inlineStr">
         <is>
-          <t>12241-RPY -G000-M</t>
+          <t>12234-RPY -G000-M</t>
         </is>
       </c>
       <c r="B139" s="4" t="inlineStr">
         <is>
-          <t>RPY Cam Holder Ex #1 (machined)</t>
+          <t>RPY Cam Holder In #4 (machined)</t>
         </is>
       </c>
       <c r="C139" s="4" t="inlineStr">
@@ -9790,19 +9790,19 @@
       </c>
       <c r="Q139" s="4" t="inlineStr">
         <is>
-          <t>Machined identity minted by Machining OUT from 12241-RPY -G000.</t>
+          <t>Machined identity minted by Machining OUT from 12234-RPY -G000.</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="4" t="inlineStr">
         <is>
-          <t>12242-RPY -G000-M</t>
+          <t>12235-RPY -G000-M</t>
         </is>
       </c>
       <c r="B140" s="4" t="inlineStr">
         <is>
-          <t>RPY Cam Holder Ex #2 (machined)</t>
+          <t>RPY Cam Holder In #5 (machined)</t>
         </is>
       </c>
       <c r="C140" s="4" t="inlineStr">
@@ -9857,19 +9857,19 @@
       </c>
       <c r="Q140" s="4" t="inlineStr">
         <is>
-          <t>Machined identity minted by Machining OUT from 12242-RPY -G000.</t>
+          <t>Machined identity minted by Machining OUT from 12235-RPY -G000.</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="4" t="inlineStr">
         <is>
-          <t>12243-RPY -G000-M</t>
+          <t>12241-RPY -G000-M</t>
         </is>
       </c>
       <c r="B141" s="4" t="inlineStr">
         <is>
-          <t>RPY Cam Holder Ex #3 (machined)</t>
+          <t>RPY Cam Holder Ex #1 (machined)</t>
         </is>
       </c>
       <c r="C141" s="4" t="inlineStr">
@@ -9924,19 +9924,19 @@
       </c>
       <c r="Q141" s="4" t="inlineStr">
         <is>
-          <t>Machined identity minted by Machining OUT from 12243-RPY -G000.</t>
+          <t>Machined identity minted by Machining OUT from 12241-RPY -G000.</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="4" t="inlineStr">
         <is>
-          <t>12244-RPY -G000-M</t>
+          <t>12242-RPY -G000-M</t>
         </is>
       </c>
       <c r="B142" s="4" t="inlineStr">
         <is>
-          <t>RPY Cam Holder Ex #4 (machined)</t>
+          <t>RPY Cam Holder Ex #2 (machined)</t>
         </is>
       </c>
       <c r="C142" s="4" t="inlineStr">
@@ -9991,19 +9991,19 @@
       </c>
       <c r="Q142" s="4" t="inlineStr">
         <is>
-          <t>Machined identity minted by Machining OUT from 12244-RPY -G000.</t>
+          <t>Machined identity minted by Machining OUT from 12242-RPY -G000.</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="4" t="inlineStr">
         <is>
-          <t>12245-RPY -G000-M</t>
+          <t>12243-RPY -G000-M</t>
         </is>
       </c>
       <c r="B143" s="4" t="inlineStr">
         <is>
-          <t>RPY Cam Holder Ex #5 (machined)</t>
+          <t>RPY Cam Holder Ex #3 (machined)</t>
         </is>
       </c>
       <c r="C143" s="4" t="inlineStr">
@@ -10058,19 +10058,19 @@
       </c>
       <c r="Q143" s="4" t="inlineStr">
         <is>
-          <t>Machined identity minted by Machining OUT from 12245-RPY -G000.</t>
+          <t>Machined identity minted by Machining OUT from 12243-RPY -G000.</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="4" t="inlineStr">
         <is>
-          <t>12246-RPY -G000-M</t>
+          <t>12244-RPY -G000-M</t>
         </is>
       </c>
       <c r="B144" s="4" t="inlineStr">
         <is>
-          <t>RPY Cam Holder Ex #6 (machined)</t>
+          <t>RPY Cam Holder Ex #4 (machined)</t>
         </is>
       </c>
       <c r="C144" s="4" t="inlineStr">
@@ -10125,19 +10125,19 @@
       </c>
       <c r="Q144" s="4" t="inlineStr">
         <is>
-          <t>Machined identity minted by Machining OUT from 12246-RPY -G000.</t>
+          <t>Machined identity minted by Machining OUT from 12244-RPY -G000.</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="4" t="inlineStr">
         <is>
-          <t>12261-RPY -G000-M</t>
+          <t>12245-RPY -G000-M</t>
         </is>
       </c>
       <c r="B145" s="4" t="inlineStr">
         <is>
-          <t>RPY Rocker Shaft #1 (machined)</t>
+          <t>RPY Cam Holder Ex #5 (machined)</t>
         </is>
       </c>
       <c r="C145" s="4" t="inlineStr">
@@ -10192,19 +10192,19 @@
       </c>
       <c r="Q145" s="4" t="inlineStr">
         <is>
-          <t>Machined identity minted by Machining OUT from 12261-RPY -G000.</t>
+          <t>Machined identity minted by Machining OUT from 12245-RPY -G000.</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="4" t="inlineStr">
         <is>
-          <t>12262-RPY -G000-M</t>
+          <t>12246-RPY -G000-M</t>
         </is>
       </c>
       <c r="B146" s="4" t="inlineStr">
         <is>
-          <t>RPY Rocker Shaft #2 (machined)</t>
+          <t>RPY Cam Holder Ex #6 (machined)</t>
         </is>
       </c>
       <c r="C146" s="4" t="inlineStr">
@@ -10259,19 +10259,19 @@
       </c>
       <c r="Q146" s="4" t="inlineStr">
         <is>
-          <t>Machined identity minted by Machining OUT from 12262-RPY -G000.</t>
+          <t>Machined identity minted by Machining OUT from 12246-RPY -G000.</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="4" t="inlineStr">
         <is>
-          <t>12263-RPY -G000-M</t>
+          <t>12261-RPY -G000-M</t>
         </is>
       </c>
       <c r="B147" s="4" t="inlineStr">
         <is>
-          <t>RPY Rocker Shaft #3 (machined)</t>
+          <t>RPY Rocker Shaft #1 (machined)</t>
         </is>
       </c>
       <c r="C147" s="4" t="inlineStr">
@@ -10326,19 +10326,19 @@
       </c>
       <c r="Q147" s="4" t="inlineStr">
         <is>
-          <t>Machined identity minted by Machining OUT from 12263-RPY -G000.</t>
+          <t>Machined identity minted by Machining OUT from 12261-RPY -G000.</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="4" t="inlineStr">
         <is>
-          <t>12264-RPY -G000-M</t>
+          <t>12262-RPY -G000-M</t>
         </is>
       </c>
       <c r="B148" s="4" t="inlineStr">
         <is>
-          <t>RPY Rocker Shaft #4 (machined)</t>
+          <t>RPY Rocker Shaft #2 (machined)</t>
         </is>
       </c>
       <c r="C148" s="4" t="inlineStr">
@@ -10393,19 +10393,19 @@
       </c>
       <c r="Q148" s="4" t="inlineStr">
         <is>
-          <t>Machined identity minted by Machining OUT from 12264-RPY -G000.</t>
+          <t>Machined identity minted by Machining OUT from 12262-RPY -G000.</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="4" t="inlineStr">
         <is>
-          <t>12265-RPY -G000-M</t>
+          <t>12263-RPY -G000-M</t>
         </is>
       </c>
       <c r="B149" s="4" t="inlineStr">
         <is>
-          <t>RPY Rocker Shaft #5 (machined)</t>
+          <t>RPY Rocker Shaft #3 (machined)</t>
         </is>
       </c>
       <c r="C149" s="4" t="inlineStr">
@@ -10425,7 +10425,7 @@
       </c>
       <c r="F149" s="4" t="inlineStr">
         <is>
-          <t>RPY</t>
+          <t>RPY/5BA</t>
         </is>
       </c>
       <c r="G149" s="4" t="inlineStr">
@@ -10450,7 +10450,7 @@
       </c>
       <c r="O149" s="4" t="inlineStr">
         <is>
-          <t>MA2-RPYCAM1, MA2-RPYCAM2</t>
+          <t>MA2-RPY6B2, MA2-RPYCAM1, MA2-RPYCAM2</t>
         </is>
       </c>
       <c r="P149" s="4" t="inlineStr">
@@ -10460,19 +10460,19 @@
       </c>
       <c r="Q149" s="4" t="inlineStr">
         <is>
-          <t>Machined identity minted by Machining OUT from 12265-RPY -G000.</t>
+          <t>Machined identity minted by Machining OUT from 12263-RPY -G000.</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="4" t="inlineStr">
         <is>
-          <t>12271-RPY -G000-M</t>
+          <t>12264-RPY -G000-M</t>
         </is>
       </c>
       <c r="B150" s="4" t="inlineStr">
         <is>
-          <t>RPY Lower Cam Holder #1 (machined)</t>
+          <t>RPY Rocker Shaft #4 (machined)</t>
         </is>
       </c>
       <c r="C150" s="4" t="inlineStr">
@@ -10527,19 +10527,19 @@
       </c>
       <c r="Q150" s="4" t="inlineStr">
         <is>
-          <t>Machined identity minted by Machining OUT from 12271-RPY -G000.</t>
+          <t>Machined identity minted by Machining OUT from 12264-RPY -G000.</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="4" t="inlineStr">
         <is>
-          <t>12272-RPY -G000-M</t>
+          <t>12265-RPY -G000-M</t>
         </is>
       </c>
       <c r="B151" s="4" t="inlineStr">
         <is>
-          <t>RPY Lower Cam Holder #2 (machined)</t>
+          <t>RPY Rocker Shaft #5 (machined)</t>
         </is>
       </c>
       <c r="C151" s="4" t="inlineStr">
@@ -10559,7 +10559,7 @@
       </c>
       <c r="F151" s="4" t="inlineStr">
         <is>
-          <t>RPY/5BA</t>
+          <t>RPY</t>
         </is>
       </c>
       <c r="G151" s="4" t="inlineStr">
@@ -10584,7 +10584,7 @@
       </c>
       <c r="O151" s="4" t="inlineStr">
         <is>
-          <t>MA2-RPY6B2, MA2-RPYCAM1, MA2-RPYCAM2</t>
+          <t>MA2-RPYCAM1, MA2-RPYCAM2</t>
         </is>
       </c>
       <c r="P151" s="4" t="inlineStr">
@@ -10594,19 +10594,19 @@
       </c>
       <c r="Q151" s="4" t="inlineStr">
         <is>
-          <t>Machined identity minted by Machining OUT from 12272-RPY -G000.</t>
+          <t>Machined identity minted by Machining OUT from 12265-RPY -G000.</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="4" t="inlineStr">
         <is>
-          <t>12273-RPY -G000-M</t>
+          <t>12271-RPY -G000-M</t>
         </is>
       </c>
       <c r="B152" s="4" t="inlineStr">
         <is>
-          <t>RPY Lower Cam Holder #3 (machined)</t>
+          <t>RPY Lower Cam Holder #1 (machined)</t>
         </is>
       </c>
       <c r="C152" s="4" t="inlineStr">
@@ -10661,19 +10661,19 @@
       </c>
       <c r="Q152" s="4" t="inlineStr">
         <is>
-          <t>Machined identity minted by Machining OUT from 12273-RPY -G000.</t>
+          <t>Machined identity minted by Machining OUT from 12271-RPY -G000.</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="4" t="inlineStr">
         <is>
-          <t>12274-RPY -G000-M</t>
+          <t>12272-RPY -G000-M</t>
         </is>
       </c>
       <c r="B153" s="4" t="inlineStr">
         <is>
-          <t>RPY Lower Cam Holder #4 (machined)</t>
+          <t>RPY Lower Cam Holder #2 (machined)</t>
         </is>
       </c>
       <c r="C153" s="4" t="inlineStr">
@@ -10728,19 +10728,19 @@
       </c>
       <c r="Q153" s="4" t="inlineStr">
         <is>
-          <t>Machined identity minted by Machining OUT from 12274-RPY -G000.</t>
+          <t>Machined identity minted by Machining OUT from 12272-RPY -G000.</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="4" t="inlineStr">
         <is>
-          <t>12265-5BA -G000-M</t>
+          <t>12273-RPY -G000-M</t>
         </is>
       </c>
       <c r="B154" s="4" t="inlineStr">
         <is>
-          <t>5BA Rocker Shaft #5 (machined)</t>
+          <t>RPY Lower Cam Holder #3 (machined)</t>
         </is>
       </c>
       <c r="C154" s="4" t="inlineStr">
@@ -10760,7 +10760,7 @@
       </c>
       <c r="F154" s="4" t="inlineStr">
         <is>
-          <t>5BA</t>
+          <t>RPY/5BA</t>
         </is>
       </c>
       <c r="G154" s="4" t="inlineStr">
@@ -10785,7 +10785,7 @@
       </c>
       <c r="O154" s="4" t="inlineStr">
         <is>
-          <t>MA2-RPYCAM1, MA2-RPYCAM2</t>
+          <t>MA2-RPY6B2, MA2-RPYCAM1, MA2-RPYCAM2</t>
         </is>
       </c>
       <c r="P154" s="4" t="inlineStr">
@@ -10795,19 +10795,19 @@
       </c>
       <c r="Q154" s="4" t="inlineStr">
         <is>
-          <t>Machined identity minted by Machining OUT from 12265-5BA -G000.</t>
+          <t>Machined identity minted by Machining OUT from 12273-RPY -G000.</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="4" t="inlineStr">
         <is>
-          <t>12265-6B2 -A000-M</t>
+          <t>12274-RPY -G000-M</t>
         </is>
       </c>
       <c r="B155" s="4" t="inlineStr">
         <is>
-          <t>5BA Rocker Shaft #5 (machined)</t>
+          <t>RPY Lower Cam Holder #4 (machined)</t>
         </is>
       </c>
       <c r="C155" s="4" t="inlineStr">
@@ -10827,7 +10827,7 @@
       </c>
       <c r="F155" s="4" t="inlineStr">
         <is>
-          <t>5BA</t>
+          <t>RPY/5BA</t>
         </is>
       </c>
       <c r="G155" s="4" t="inlineStr">
@@ -10852,7 +10852,7 @@
       </c>
       <c r="O155" s="4" t="inlineStr">
         <is>
-          <t>MA2-RPYCAM1, MA2-RPYCAM2</t>
+          <t>MA2-RPY6B2, MA2-RPYCAM1, MA2-RPYCAM2</t>
         </is>
       </c>
       <c r="P155" s="4" t="inlineStr">
@@ -10862,19 +10862,19 @@
       </c>
       <c r="Q155" s="4" t="inlineStr">
         <is>
-          <t>Machined identity minted by Machining OUT from 12265-6B2 -A000.</t>
+          <t>Machined identity minted by Machining OUT from 12274-RPY -G000.</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="4" t="inlineStr">
         <is>
-          <t>12270-6NAA-M</t>
+          <t>12265-5BA -G000-M</t>
         </is>
       </c>
       <c r="B156" s="4" t="inlineStr">
         <is>
-          <t>6NA Fuel Pump Raw (machined)</t>
+          <t>5BA Rocker Shaft #5 (machined)</t>
         </is>
       </c>
       <c r="C156" s="4" t="inlineStr">
@@ -10894,7 +10894,7 @@
       </c>
       <c r="F156" s="4" t="inlineStr">
         <is>
-          <t>6NA</t>
+          <t>5BA</t>
         </is>
       </c>
       <c r="G156" s="4" t="inlineStr">
@@ -10919,7 +10919,7 @@
       </c>
       <c r="O156" s="4" t="inlineStr">
         <is>
-          <t>MA1-FP6NA</t>
+          <t>MA2-RPYCAM1, MA2-RPYCAM2</t>
         </is>
       </c>
       <c r="P156" s="4" t="inlineStr">
@@ -10929,19 +10929,19 @@
       </c>
       <c r="Q156" s="4" t="inlineStr">
         <is>
-          <t>Machined identity minted by Machining OUT from 12270-6NAA.</t>
+          <t>Machined identity minted by Machining OUT from 12265-5BA -G000.</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="4" t="inlineStr">
         <is>
-          <t>12270-6VJA-M</t>
+          <t>12265-6B2 -A000-M</t>
         </is>
       </c>
       <c r="B157" s="4" t="inlineStr">
         <is>
-          <t>6VJ Fuel Pump Raw (machined)</t>
+          <t>5BA Rocker Shaft #5 (machined)</t>
         </is>
       </c>
       <c r="C157" s="4" t="inlineStr">
@@ -10961,7 +10961,7 @@
       </c>
       <c r="F157" s="4" t="inlineStr">
         <is>
-          <t>6VJ</t>
+          <t>5BA</t>
         </is>
       </c>
       <c r="G157" s="4" t="inlineStr">
@@ -10986,7 +10986,7 @@
       </c>
       <c r="O157" s="4" t="inlineStr">
         <is>
-          <t>MA1-FP6NA</t>
+          <t>MA2-RPYCAM1, MA2-RPYCAM2</t>
         </is>
       </c>
       <c r="P157" s="4" t="inlineStr">
@@ -10996,19 +10996,19 @@
       </c>
       <c r="Q157" s="4" t="inlineStr">
         <is>
-          <t>Machined identity minted by Machining OUT from 12270-6VJA.</t>
+          <t>Machined identity minted by Machining OUT from 12265-6B2 -A000.</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="4" t="inlineStr">
         <is>
-          <t>12270-5PAA-M</t>
+          <t>12270-6NAA-M</t>
         </is>
       </c>
       <c r="B158" s="4" t="inlineStr">
         <is>
-          <t>5PA Fuel Pump Raw (machined)</t>
+          <t>6NA Fuel Pump Raw (machined)</t>
         </is>
       </c>
       <c r="C158" s="4" t="inlineStr">
@@ -11028,7 +11028,7 @@
       </c>
       <c r="F158" s="4" t="inlineStr">
         <is>
-          <t>5PA</t>
+          <t>6NA</t>
         </is>
       </c>
       <c r="G158" s="4" t="inlineStr">
@@ -11053,7 +11053,7 @@
       </c>
       <c r="O158" s="4" t="inlineStr">
         <is>
-          <t>MA2-5PA</t>
+          <t>MA1-FP6NA</t>
         </is>
       </c>
       <c r="P158" s="4" t="inlineStr">
@@ -11063,19 +11063,19 @@
       </c>
       <c r="Q158" s="4" t="inlineStr">
         <is>
-          <t>Machined identity minted by Machining OUT from 12270-5PAA.</t>
+          <t>Machined identity minted by Machining OUT from 12270-6NAA.</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="4" t="inlineStr">
         <is>
-          <t>12270-6B2A-M</t>
+          <t>12270-6VJA-M</t>
         </is>
       </c>
       <c r="B159" s="4" t="inlineStr">
         <is>
-          <t>6B2 Fuel Pump Raw (machined)</t>
+          <t>6VJ Fuel Pump Raw (machined)</t>
         </is>
       </c>
       <c r="C159" s="4" t="inlineStr">
@@ -11095,7 +11095,7 @@
       </c>
       <c r="F159" s="4" t="inlineStr">
         <is>
-          <t>6B2</t>
+          <t>6VJ</t>
         </is>
       </c>
       <c r="G159" s="4" t="inlineStr">
@@ -11120,22 +11120,156 @@
       </c>
       <c r="O159" s="4" t="inlineStr">
         <is>
+          <t>MA1-FP6NA</t>
+        </is>
+      </c>
+      <c r="P159" s="4" t="inlineStr">
+        <is>
+          <t>SYNTHESIZED</t>
+        </is>
+      </c>
+      <c r="Q159" s="4" t="inlineStr">
+        <is>
+          <t>Machined identity minted by Machining OUT from 12270-6VJA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="4" t="inlineStr">
+        <is>
+          <t>12270-5PAA-M</t>
+        </is>
+      </c>
+      <c r="B160" s="4" t="inlineStr">
+        <is>
+          <t>5PA Fuel Pump Raw (machined)</t>
+        </is>
+      </c>
+      <c r="C160" s="4" t="inlineStr">
+        <is>
+          <t>SubAssembly</t>
+        </is>
+      </c>
+      <c r="D160" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E160" s="4" t="inlineStr">
+        <is>
+          <t>Machined</t>
+        </is>
+      </c>
+      <c r="F160" s="4" t="inlineStr">
+        <is>
+          <t>5PA</t>
+        </is>
+      </c>
+      <c r="G160" s="4" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="H160" s="4" t="inlineStr"/>
+      <c r="I160" s="4" t="inlineStr"/>
+      <c r="J160" s="4" t="inlineStr"/>
+      <c r="K160" s="4" t="inlineStr"/>
+      <c r="L160" s="4" t="inlineStr"/>
+      <c r="M160" s="4" t="inlineStr">
+        <is>
+          <t>Blue Ridge (synthesized)</t>
+        </is>
+      </c>
+      <c r="N160" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O160" s="4" t="inlineStr">
+        <is>
+          <t>MA2-5PA</t>
+        </is>
+      </c>
+      <c r="P160" s="4" t="inlineStr">
+        <is>
+          <t>SYNTHESIZED</t>
+        </is>
+      </c>
+      <c r="Q160" s="4" t="inlineStr">
+        <is>
+          <t>Machined identity minted by Machining OUT from 12270-5PAA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="4" t="inlineStr">
+        <is>
+          <t>12270-6B2A-M</t>
+        </is>
+      </c>
+      <c r="B161" s="4" t="inlineStr">
+        <is>
+          <t>6B2 Fuel Pump Raw (machined)</t>
+        </is>
+      </c>
+      <c r="C161" s="4" t="inlineStr">
+        <is>
+          <t>SubAssembly</t>
+        </is>
+      </c>
+      <c r="D161" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E161" s="4" t="inlineStr">
+        <is>
+          <t>Machined</t>
+        </is>
+      </c>
+      <c r="F161" s="4" t="inlineStr">
+        <is>
+          <t>6B2</t>
+        </is>
+      </c>
+      <c r="G161" s="4" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="H161" s="4" t="inlineStr"/>
+      <c r="I161" s="4" t="inlineStr"/>
+      <c r="J161" s="4" t="inlineStr"/>
+      <c r="K161" s="4" t="inlineStr"/>
+      <c r="L161" s="4" t="inlineStr"/>
+      <c r="M161" s="4" t="inlineStr">
+        <is>
+          <t>Blue Ridge (synthesized)</t>
+        </is>
+      </c>
+      <c r="N161" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O161" s="4" t="inlineStr">
+        <is>
           <t>MA2-RPY6B2</t>
         </is>
       </c>
-      <c r="P159" s="4" t="inlineStr">
+      <c r="P161" s="4" t="inlineStr">
         <is>
           <t>SYNTHESIZED</t>
         </is>
       </c>
-      <c r="Q159" s="4" t="inlineStr">
+      <c r="Q161" s="4" t="inlineStr">
         <is>
           <t>Machined identity minted by Machining OUT from 12270-6B2A.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q159"/>
+  <autoFilter ref="A1:Q161"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -39243,7 +39377,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J33"/>
+  <dimension ref="A1:J35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -40169,7 +40303,7 @@
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>19320-6A0 -A510</t>
+          <t>19320-6A0 -A510-AEP</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
@@ -40207,22 +40341,22 @@
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>19410-6A0 -A000</t>
+          <t>19320-6A0 -A510-ISP</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>6A0 Water Passage (AEP)</t>
+          <t>6A0 Thermo Case Auto (ISP)</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>16</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E25" s="3" t="n">
@@ -40245,22 +40379,22 @@
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>19321-64S -A000</t>
+          <t>19410-6A0 -A000-AEP</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>64S Thermo Case</t>
+          <t>6A0 Water Passage (AEP)</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>60</t>
         </is>
       </c>
       <c r="E26" s="3" t="n">
@@ -40283,22 +40417,22 @@
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>12270-6MA -J000</t>
+          <t>19410-6A0 -A000-ISP</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>6MA Fuel Pump</t>
+          <t>6A0 Water Passage (ISP)</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>12</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E27" s="3" t="n">
@@ -40321,12 +40455,12 @@
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>19321-66V -A000</t>
+          <t>19321-64S -A000</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>66V Thermo Case</t>
+          <t>64S Thermo Case</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
@@ -40359,12 +40493,12 @@
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>12270-6MD -A000</t>
+          <t>12270-6MA -J000</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>6MD Fuel Pump</t>
+          <t>6MA Fuel Pump</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
@@ -40395,62 +40529,62 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>14850-6MD -A000</t>
-        </is>
-      </c>
-      <c r="B30" s="2" t="inlineStr">
-        <is>
-          <t>6MD Oil Jet</t>
-        </is>
-      </c>
-      <c r="C30" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D30" s="2" t="inlineStr">
-        <is>
-          <t>60</t>
-        </is>
-      </c>
-      <c r="E30" s="2" t="n">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>19321-66V -A000</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>66V Thermo Case</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="F30" s="2" t="inlineStr">
-        <is>
-          <t>ByVision</t>
-        </is>
-      </c>
-      <c r="G30" s="2" t="inlineStr"/>
-      <c r="H30" s="2" t="inlineStr"/>
-      <c r="I30" s="2" t="inlineStr"/>
-      <c r="J30" s="2" t="inlineStr">
-        <is>
-          <t>Camera</t>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>ByWeight</t>
+        </is>
+      </c>
+      <c r="G30" s="3" t="inlineStr"/>
+      <c r="H30" s="3" t="inlineStr"/>
+      <c r="I30" s="3" t="inlineStr"/>
+      <c r="J30" s="3" t="inlineStr">
+        <is>
+          <t>Scale</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>19410-6MD -A000</t>
+          <t>12270-6MD -A000</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>6MD Water Passage</t>
+          <t>6MD Fuel Pump</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>24</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E31" s="3" t="n">
@@ -40471,62 +40605,62 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="3" t="inlineStr">
-        <is>
-          <t>12230-P8A -A000</t>
-        </is>
-      </c>
-      <c r="B32" s="3" t="inlineStr">
-        <is>
-          <t>Cam Thrust Front</t>
-        </is>
-      </c>
-      <c r="C32" s="3" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="D32" s="3" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
-      </c>
-      <c r="E32" s="3" t="n">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>14850-6MD -A000</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>6MD Oil Jet</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="F32" s="3" t="inlineStr">
-        <is>
-          <t>ByWeight</t>
-        </is>
-      </c>
-      <c r="G32" s="3" t="inlineStr"/>
-      <c r="H32" s="3" t="inlineStr"/>
-      <c r="I32" s="3" t="inlineStr"/>
-      <c r="J32" s="3" t="inlineStr">
-        <is>
-          <t>Scale</t>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>ByVision</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr"/>
+      <c r="H32" s="2" t="inlineStr"/>
+      <c r="I32" s="2" t="inlineStr"/>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>Camera</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>19321-66V-A100</t>
+          <t>19410-6MD -A000</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>66V Thermo Case</t>
+          <t>6MD Water Passage</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>60</t>
         </is>
       </c>
       <c r="E33" s="3" t="n">
@@ -40546,8 +40680,84 @@
         </is>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>12230-P8A -A000</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>Cam Thrust Front</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>ByWeight</t>
+        </is>
+      </c>
+      <c r="G34" s="3" t="inlineStr"/>
+      <c r="H34" s="3" t="inlineStr"/>
+      <c r="I34" s="3" t="inlineStr"/>
+      <c r="J34" s="3" t="inlineStr">
+        <is>
+          <t>Scale</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>19321-66V-A100</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>66V Thermo Case</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F35" s="3" t="inlineStr">
+        <is>
+          <t>ByWeight</t>
+        </is>
+      </c>
+      <c r="G35" s="3" t="inlineStr"/>
+      <c r="H35" s="3" t="inlineStr"/>
+      <c r="I35" s="3" t="inlineStr"/>
+      <c r="J35" s="3" t="inlineStr">
+        <is>
+          <t>Scale</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J33"/>
+  <autoFilter ref="A1:J35"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -40558,7 +40768,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -40700,7 +40910,7 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>19320-6A0 -A510</t>
+          <t>19320-6A0 -A510-AEP</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -40715,7 +40925,7 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>6AO/6A0</t>
+          <t>6AO</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
@@ -40732,12 +40942,12 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>19410-6A0 -A000</t>
+          <t>19320-6A0 -A510-ISP</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>6A0 Water Passage (AEP)</t>
+          <t>6A0 Thermo Case Auto (ISP)</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
@@ -40764,12 +40974,12 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>19321-64S -A000</t>
+          <t>19410-6A0 -A000-AEP</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>64S Thermo Case</t>
+          <t>6A0 Water Passage (AEP)</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
@@ -40779,7 +40989,7 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>64S</t>
+          <t>6A0</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
@@ -40796,12 +41006,12 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>12270-6MA -J000</t>
+          <t>19410-6A0 -A000-ISP</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>6MA Fuel Pump</t>
+          <t>6A0 Water Passage (ISP)</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
@@ -40811,7 +41021,7 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>6MA</t>
+          <t>6A0</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
@@ -40828,12 +41038,12 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>19321-66V -A000</t>
+          <t>19321-64S -A000</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>66V Thermo Case</t>
+          <t>64S Thermo Case</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
@@ -40843,7 +41053,7 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>66V</t>
+          <t>64S</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
@@ -40860,12 +41070,12 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>12270-6MD -A000</t>
+          <t>12270-6MA -J000</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>6MD Fuel Pump</t>
+          <t>6MA Fuel Pump</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
@@ -40875,7 +41085,7 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>6MD</t>
+          <t>6MA</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
@@ -40892,12 +41102,12 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>14850-6MD -A000</t>
+          <t>19321-66V -A000</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>6MD Oil Jet</t>
+          <t>66V Thermo Case</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
@@ -40907,7 +41117,7 @@
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>6MD</t>
+          <t>66V</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
@@ -40924,12 +41134,12 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>19410-6MD -A000</t>
+          <t>12270-6MD -A000</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>6MD Water Passage</t>
+          <t>6MD Fuel Pump</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
@@ -40956,12 +41166,12 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>12230-P8A -A000</t>
+          <t>14850-6MD -A000</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Cam Thrust Front</t>
+          <t>6MD Oil Jet</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
@@ -40971,7 +41181,7 @@
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>P8A</t>
+          <t>6MD</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
@@ -40988,37 +41198,101 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
+          <t>19410-6MD -A000</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>6MD Water Passage</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>FinishedGood</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>6MD</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>Off-Site</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>Off-site part - manufactured away from Madison; no MPP line applies.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>12230-P8A -A000</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Cam Thrust Front</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>FinishedGood</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>P8A</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>Off-Site</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>Off-site part - manufactured away from Madison; no MPP line applies.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
           <t>19321-66V-A100</t>
         </is>
       </c>
-      <c r="B14" s="3" t="inlineStr">
+      <c r="B16" s="3" t="inlineStr">
         <is>
           <t>66V Thermo Case</t>
         </is>
       </c>
-      <c r="C14" s="3" t="inlineStr">
+      <c r="C16" s="3" t="inlineStr">
         <is>
           <t>FinishedGood</t>
         </is>
       </c>
-      <c r="D14" s="3" t="inlineStr">
+      <c r="D16" s="3" t="inlineStr">
         <is>
           <t>66V</t>
         </is>
       </c>
-      <c r="E14" s="3" t="inlineStr">
+      <c r="E16" s="3" t="inlineStr">
         <is>
           <t>Off-Site</t>
         </is>
       </c>
-      <c r="F14" s="3" t="inlineStr">
+      <c r="F16" s="3" t="inlineStr">
         <is>
           <t>Off-site part - manufactured away from Madison; no MPP line applies.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F14"/>
+  <autoFilter ref="A1:F16"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -41029,7 +41303,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E65"/>
+  <dimension ref="A1:E67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -41371,22 +41645,22 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Packaging</t>
+          <t>Parts</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>19320-6A0 -A510</t>
+          <t>1223A-6B2 -A000</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>Second packaging row for the same part (16 trays x 6 parts, Scale).</t>
+          <t>MPP typed this "Component", but it is a BOM parent with 22 components - it is an assembled part, not a raw one.</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>UQ_ContainerConfig_ActiveItemId permits one active config. Row dropped; MPP must split the part number or pick one rule.</t>
+          <t>Treated as assembled (no die-cast route, no machined identity). MPP should re-type it as FinishedGood.</t>
         </is>
       </c>
     </row>
@@ -41398,130 +41672,130 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Packaging</t>
+          <t>Parts</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>19410-6A0 -A000</t>
+          <t>19321-66V -A000 / 19321-66V-A100</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>Second packaging row for the same part (12 trays x 15 parts, Scale).</t>
+          <t>Two part numbers with the identical description "66V Thermo Case".</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>UQ_ContainerConfig_ActiveItemId permits one active config. Row dropped; MPP must split the part number or pick one rule.</t>
+          <t>Loaded as two items. MPP to confirm both are live, or retire one.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>Parts</t>
-        </is>
-      </c>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t>1223A-6B2 -A000</t>
-        </is>
-      </c>
-      <c r="D15" s="3" t="inlineStr">
-        <is>
-          <t>MPP typed this "Component", but it is a BOM parent with 22 components - it is an assembled part, not a raw one.</t>
-        </is>
-      </c>
-      <c r="E15" s="3" t="inlineStr">
-        <is>
-          <t>Treated as assembled (no die-cast route, no machined identity). MPP should re-type it as FinishedGood.</t>
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>BOM</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>11200-6FB-A000</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>Component "6FB Oil Pan Raw" appears in no BOM, so its line was inferred from program 6FB, which covers 2 finished goods.</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>Eligible at all of them: MA2-6FBCHOP. MPP should supply the BOM.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="B16" s="3" t="inlineStr">
-        <is>
-          <t>Parts</t>
-        </is>
-      </c>
-      <c r="C16" s="3" t="inlineStr">
-        <is>
-          <t>19320-6A0 -A510</t>
-        </is>
-      </c>
-      <c r="D16" s="3" t="inlineStr">
-        <is>
-          <t>One part number used for two different parts: 6A0 Thermo Case Auto (AEP) (basket 5); 6A0 Thermo Case Auto (ISP) (basket 6).</t>
-        </is>
-      </c>
-      <c r="E16" s="3" t="inlineStr">
-        <is>
-          <t>UQ_Item_PartNumber allows one row. MPP must supply a distinct number for the second variant, or confirm they are the same part.</t>
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>BOM</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>12270-6B2 -A000 -&gt; 92900-06012-0B</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>BOM note says "10x12 Dowel Pin" but the part is "6x12 Stud Bolt".</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>Item description kept. MPP to confirm the correct component.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>Parts</t>
-        </is>
-      </c>
-      <c r="C17" s="3" t="inlineStr">
-        <is>
-          <t>19321-66V -A000 / 19321-66V-A100</t>
-        </is>
-      </c>
-      <c r="D17" s="3" t="inlineStr">
-        <is>
-          <t>Two part numbers with the identical description "66V Thermo Case".</t>
-        </is>
-      </c>
-      <c r="E17" s="3" t="inlineStr">
-        <is>
-          <t>Loaded as two items. MPP to confirm both are live, or retire one.</t>
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>BOM</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>90009-R70-A000</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>Component "14mm Bolt Plug" appears in no BOM, so its line was inferred from program 6FB/5J6-1, which covers 3 finished goods.</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>Eligible at all of them: MA2-6FBCHOP, MA2-V6OP. MPP should supply the BOM.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="B18" s="3" t="inlineStr">
-        <is>
-          <t>Parts</t>
-        </is>
-      </c>
-      <c r="C18" s="3" t="inlineStr">
-        <is>
-          <t>19410-6A0 -A000</t>
-        </is>
-      </c>
-      <c r="D18" s="3" t="inlineStr">
-        <is>
-          <t>One part number used for two different parts: 6A0 Water Passage (AEP) (basket 60); 6A0 Water Passage (ISP) (basket 15).</t>
-        </is>
-      </c>
-      <c r="E18" s="3" t="inlineStr">
-        <is>
-          <t>UQ_Item_PartNumber allows one row. MPP must supply a distinct number for the second variant, or confirm they are the same part.</t>
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>BOM</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>94301-08140</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>Component "8x14 Dowel Pin" appears in no BOM, so its line was inferred from program 6FB/5J6-1, which covers 3 finished goods.</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>Eligible at all of them: MA2-6FBCHOP, MA2-V6OP. MPP should supply the BOM.</t>
         </is>
       </c>
     </row>
@@ -41533,22 +41807,22 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>BOM</t>
+          <t>Locations</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>11200-6FB-A000</t>
+          <t>66B-TC</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>Component "6FB Oil Pan Raw" appears in no BOM, so its line was inferred from program 6FB, which covers 2 finished goods.</t>
+          <t>Configured production line "66B Thermal Case" has no part assigned to it.</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>Eligible at all of them: MA2-6FBCHOP. MPP should supply the BOM.</t>
+          <t>Either MPP omitted its parts, or the line is idle.</t>
         </is>
       </c>
     </row>
@@ -41560,22 +41834,22 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>BOM</t>
+          <t>Locations</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>12270-6B2 -A000 -&gt; 92900-06012-0B</t>
+          <t>AO-OP</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>BOM note says "10x12 Dowel Pin" but the part is "6x12 Stud Bolt".</t>
+          <t>Configured production line "Assembly Out Oil Passage" has no part assigned to it.</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>Item description kept. MPP to confirm the correct component.</t>
+          <t>Either MPP omitted its parts, or the line is idle.</t>
         </is>
       </c>
     </row>
@@ -41587,22 +41861,22 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>BOM</t>
+          <t>Locations</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>90009-R70-A000</t>
+          <t>MA1-COMPBR</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>Component "14mm Bolt Plug" appears in no BOM, so its line was inferred from program 6FB/5J6-1, which covers 3 finished goods.</t>
+          <t>Configured production line "RPY Comp bracket" has no part assigned to it.</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>Eligible at all of them: MA2-6FBCHOP, MA2-V6OP. MPP should supply the BOM.</t>
+          <t>Either MPP omitted its parts, or the line is idle.</t>
         </is>
       </c>
     </row>
@@ -41614,22 +41888,22 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>BOM</t>
+          <t>Locations</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>94301-08140</t>
+          <t>MA2-COS</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>Component "8x14 Dowel Pin" appears in no BOM, so its line was inferred from program 6FB/5J6-1, which covers 3 finished goods.</t>
+          <t>Configured production line "Case Oil Seal" has no part assigned to it.</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>Eligible at all of them: MA2-6FBCHOP, MA2-V6OP. MPP should supply the BOM.</t>
+          <t>Either MPP omitted its parts, or the line is idle.</t>
         </is>
       </c>
     </row>
@@ -41641,22 +41915,22 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Locations</t>
+          <t>Packaging</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>66B-TC</t>
+          <t>12230-P8A -A000</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>Configured production line "66B Thermal Case" has no part assigned to it.</t>
+          <t>Closure is "Scale" (ByWeight) but no Target Weight was given.</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>Either MPP omitted its parts, or the line is idle.</t>
+          <t>TargetWeight left NULL - the scale close cannot validate without it.</t>
         </is>
       </c>
     </row>
@@ -41668,22 +41942,22 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>Locations</t>
+          <t>Packaging</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>AO-OP</t>
+          <t>1223A-59B -A0002</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>Configured production line "Assembly Out Oil Passage" has no part assigned to it.</t>
+          <t>Blue Ridge dev-seed part number appears in the customer workbook.</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>Either MPP omitted its parts, or the line is idle.</t>
+          <t>Row dropped - not an MPP part.</t>
         </is>
       </c>
     </row>
@@ -41695,22 +41969,22 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>Locations</t>
+          <t>Packaging</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>MA1-COMPBR</t>
+          <t>12270-6MA -J000</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>Configured production line "RPY Comp bracket" has no part assigned to it.</t>
+          <t>Closure is "Scale" (ByWeight) but no Target Weight was given.</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>Either MPP omitted its parts, or the line is idle.</t>
+          <t>TargetWeight left NULL - the scale close cannot validate without it.</t>
         </is>
       </c>
     </row>
@@ -41722,22 +41996,22 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>Locations</t>
+          <t>Packaging</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>MA2-COS</t>
+          <t>12270-6MD -A000</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>Configured production line "Case Oil Seal" has no part assigned to it.</t>
+          <t>Closure is "Scale" (ByWeight) but no Target Weight was given.</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>Either MPP omitted its parts, or the line is idle.</t>
+          <t>TargetWeight left NULL - the scale close cannot validate without it.</t>
         </is>
       </c>
     </row>
@@ -41754,7 +42028,7 @@
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>12230-P8A -A000</t>
+          <t>14650-5GO -A000</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
@@ -41781,17 +42055,17 @@
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>1223A-59B -A0002</t>
+          <t>14660-5GO -A000</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>Blue Ridge dev-seed part number appears in the customer workbook.</t>
+          <t>Closure is "Scale" (ByWeight) but no Target Weight was given.</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>Row dropped - not an MPP part.</t>
+          <t>TargetWeight left NULL - the scale close cannot validate without it.</t>
         </is>
       </c>
     </row>
@@ -41808,7 +42082,7 @@
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>12270-6MA -J000</t>
+          <t>17145-6MD -A000</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
@@ -41835,7 +42109,7 @@
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>12270-6MD -A000</t>
+          <t>19320-6A0 -A010</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
@@ -41862,7 +42136,7 @@
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>14650-5GO -A000</t>
+          <t>19320-6A0 -A510-AEP</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
@@ -41889,7 +42163,7 @@
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>14660-5GO -A000</t>
+          <t>19320-6A0 -A510-ISP</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
@@ -41916,7 +42190,7 @@
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>17145-6MD -A000</t>
+          <t>19321-64S -A000</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
@@ -41943,7 +42217,7 @@
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>19320-6A0 -A010</t>
+          <t>19321-66V -A000</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
@@ -41970,7 +42244,7 @@
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>19320-6A0 -A510</t>
+          <t>19321-66V-A100</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
@@ -41997,7 +42271,7 @@
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>19321-64S -A000</t>
+          <t>1932A-69F -A000</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
@@ -42024,7 +42298,7 @@
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>19321-66V -A000</t>
+          <t>19410-6A0 -A000-AEP</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
@@ -42051,7 +42325,7 @@
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>19321-66V-A100</t>
+          <t>19410-6A0 -A000-ISP</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr">
@@ -42078,7 +42352,7 @@
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>1932A-69F -A000</t>
+          <t>19410-6MD -A000</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
@@ -42105,7 +42379,7 @@
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>19410-6A0 -A000</t>
+          <t>22533-RJ2 -0000</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
@@ -42132,17 +42406,17 @@
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>19410-6MD -A000</t>
+          <t>5G0-FG</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>Closure is "Scale" (ByWeight) but no Target Weight was given.</t>
+          <t>Blue Ridge dev-seed part number appears in the customer workbook.</t>
         </is>
       </c>
       <c r="E41" s="4" t="inlineStr">
         <is>
-          <t>TargetWeight left NULL - the scale close cannot validate without it.</t>
+          <t>Row dropped - not an MPP part.</t>
         </is>
       </c>
     </row>
@@ -42154,22 +42428,22 @@
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>Packaging</t>
+          <t>Parts</t>
         </is>
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>22533-RJ2 -0000</t>
+          <t>11221-64AA-A010</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>Closure is "Scale" (ByWeight) but no Target Weight was given.</t>
+          <t>Cannot tell from the data whether "Baffle Plate A" is die cast at MPP or purchased (shafts / baffle plates are commonly bought-in steel).</t>
         </is>
       </c>
       <c r="E42" s="4" t="inlineStr">
         <is>
-          <t>TargetWeight left NULL - the scale close cannot validate without it.</t>
+          <t>Classified as Cast. This drives the die-cast route + DC1/TRIM eligibility, so MPP should confirm.</t>
         </is>
       </c>
     </row>
@@ -42181,22 +42455,22 @@
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>Packaging</t>
+          <t>Parts</t>
         </is>
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>5G0-FG</t>
+          <t>11222-64A-A001</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
         <is>
-          <t>Blue Ridge dev-seed part number appears in the customer workbook.</t>
+          <t>Cannot tell from the data whether "Baffle Plate B" is die cast at MPP or purchased (shafts / baffle plates are commonly bought-in steel).</t>
         </is>
       </c>
       <c r="E43" s="4" t="inlineStr">
         <is>
-          <t>Row dropped - not an MPP part.</t>
+          <t>Classified as Cast. This drives the die-cast route + DC1/TRIM eligibility, so MPP should confirm.</t>
         </is>
       </c>
     </row>
@@ -42213,12 +42487,12 @@
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>11221-64AA-A010</t>
+          <t>146315GO A000</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>Cannot tell from the data whether "Baffle Plate A" is die cast at MPP or purchased (shafts / baffle plates are commonly bought-in steel).</t>
+          <t>Cannot tell from the data whether "Front In Shaft" is die cast at MPP or purchased (shafts / baffle plates are commonly bought-in steel).</t>
         </is>
       </c>
       <c r="E44" s="4" t="inlineStr">
@@ -42240,12 +42514,12 @@
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>11222-64A-A001</t>
+          <t>146325GO A000</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>Cannot tell from the data whether "Baffle Plate B" is die cast at MPP or purchased (shafts / baffle plates are commonly bought-in steel).</t>
+          <t>Cannot tell from the data whether "Front Ex Shaft" is die cast at MPP or purchased (shafts / baffle plates are commonly bought-in steel).</t>
         </is>
       </c>
       <c r="E45" s="4" t="inlineStr">
@@ -42267,12 +42541,12 @@
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>146315GO A000</t>
+          <t>146335GO A000</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr">
         <is>
-          <t>Cannot tell from the data whether "Front In Shaft" is die cast at MPP or purchased (shafts / baffle plates are commonly bought-in steel).</t>
+          <t>Cannot tell from the data whether "Rear In Shaft" is die cast at MPP or purchased (shafts / baffle plates are commonly bought-in steel).</t>
         </is>
       </c>
       <c r="E46" s="4" t="inlineStr">
@@ -42294,12 +42568,12 @@
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>146325GO A000</t>
+          <t>146345GO A000</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>Cannot tell from the data whether "Front Ex Shaft" is die cast at MPP or purchased (shafts / baffle plates are commonly bought-in steel).</t>
+          <t>Cannot tell from the data whether "Rear Ex Shaft" is die cast at MPP or purchased (shafts / baffle plates are commonly bought-in steel).</t>
         </is>
       </c>
       <c r="E47" s="4" t="inlineStr">
@@ -42321,17 +42595,17 @@
       </c>
       <c r="C48" s="4" t="inlineStr">
         <is>
-          <t>146335GO A000</t>
+          <t>19320-6A0 -A510</t>
         </is>
       </c>
       <c r="D48" s="4" t="inlineStr">
         <is>
-          <t>Cannot tell from the data whether "Rear In Shaft" is die cast at MPP or purchased (shafts / baffle plates are commonly bought-in steel).</t>
+          <t>One part number used for two different parts: 6A0 Thermo Case Auto (AEP) (basket 5); 6A0 Thermo Case Auto (ISP) (basket 6).</t>
         </is>
       </c>
       <c r="E48" s="4" t="inlineStr">
         <is>
-          <t>Classified as Cast. This drives the die-cast route + DC1/TRIM eligibility, so MPP should confirm.</t>
+          <t>Split into 19320-6A0 -A510-AEP, 19320-6A0 -A510-ISP. The suffix is a Blue Ridge convention, NOT an MPP part number, and MUST be stripped before the value reaches AIM -- Parts.ufn_AimCustomerPartNumber currently only strips dashes, so it would emit e.g. "193206A0 A510AEP". MPP should still confirm whether a real distinct number exists.</t>
         </is>
       </c>
     </row>
@@ -42348,17 +42622,17 @@
       </c>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t>146345GO A000</t>
+          <t>19410-6A0 -A000</t>
         </is>
       </c>
       <c r="D49" s="4" t="inlineStr">
         <is>
-          <t>Cannot tell from the data whether "Rear Ex Shaft" is die cast at MPP or purchased (shafts / baffle plates are commonly bought-in steel).</t>
+          <t>One part number used for two different parts: 6A0 Water Passage (AEP) (basket 60); 6A0 Water Passage (ISP) (basket 15).</t>
         </is>
       </c>
       <c r="E49" s="4" t="inlineStr">
         <is>
-          <t>Classified as Cast. This drives the die-cast route + DC1/TRIM eligibility, so MPP should confirm.</t>
+          <t>Split into 19410-6A0 -A000-AEP, 19410-6A0 -A000-ISP. The suffix is a Blue Ridge convention, NOT an MPP part number, and MUST be stripped before the value reaches AIM -- Parts.ufn_AimCustomerPartNumber currently only strips dashes, so it would emit e.g. "193206A0 A510AEP". MPP should still confirm whether a real distinct number exists.</t>
         </is>
       </c>
     </row>
@@ -42618,7 +42892,7 @@
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>19320-6A0 -A510</t>
+          <t>19320-6A0 -A510-AEP</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
@@ -42645,7 +42919,7 @@
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>19321-64S -A000</t>
+          <t>19320-6A0 -A510-ISP</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
@@ -42672,7 +42946,7 @@
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>19321-66V -A000</t>
+          <t>19321-64S -A000</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
@@ -42699,7 +42973,7 @@
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>19321-66V-A100</t>
+          <t>19321-66V -A000</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
@@ -42726,7 +43000,7 @@
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>19410-6A0 -A000</t>
+          <t>19321-66V-A100</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
@@ -42753,7 +43027,7 @@
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>19410-6MD -A000</t>
+          <t>19410-6A0 -A000-AEP</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
@@ -42780,22 +43054,76 @@
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
+          <t>19410-6A0 -A000-ISP</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>Finished good has no BOM rows.</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="inlineStr">
+        <is>
+          <t>Off-site part - no BOM expected.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>BOM</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>19410-6MD -A000</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>Finished good has no BOM rows.</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>Off-site part - no BOM expected.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>BOM</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
           <t>22533-RJ2 -0000</t>
         </is>
       </c>
-      <c r="D65" s="2" t="inlineStr">
+      <c r="D67" s="2" t="inlineStr">
         <is>
           <t>Finished good has no BOM rows.</t>
         </is>
       </c>
-      <c r="E65" s="2" t="inlineStr">
+      <c r="E67" s="2" t="inlineStr">
         <is>
           <t>Off-site part - no BOM expected.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E65"/>
+  <autoFilter ref="A1:E67"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>